<commit_message>
Update lineup from spreadsheet — add T4 and Skeptiq (Groove2Funk, Friday)
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/The FullMoon Festival Linup.xlsx
+++ b/The FullMoon Festival Linup.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1212" uniqueCount="237">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1220" uniqueCount="238">
   <si>
     <t>THE FULLMOON FESTIVAL</t>
   </si>
@@ -630,6 +630,9 @@
   </si>
   <si>
     <t>T4</t>
+  </si>
+  <si>
+    <t>Skeptiq</t>
   </si>
   <si>
     <t>Alan Stacey / Ste Butt</t>
@@ -3953,7 +3956,7 @@
     </row>
     <row r="24">
       <c r="A24" s="1" t="s">
-        <v>44</v>
+        <v>205</v>
       </c>
       <c r="B24" s="1" t="s">
         <v>28</v>
@@ -3962,10 +3965,10 @@
         <v>29</v>
       </c>
       <c r="D24" s="5">
-        <v>0.8958333333333334</v>
+        <v>0.8125</v>
       </c>
       <c r="E24" s="5">
-        <v>0.9375</v>
+        <v>0.8541666666666666</v>
       </c>
       <c r="F24" s="1" t="s">
         <v>198</v>
@@ -3973,7 +3976,7 @@
     </row>
     <row r="25">
       <c r="A25" s="1" t="s">
-        <v>47</v>
+        <v>206</v>
       </c>
       <c r="B25" s="1" t="s">
         <v>28</v>
@@ -3982,10 +3985,10 @@
         <v>29</v>
       </c>
       <c r="D25" s="5">
-        <v>0.9375</v>
+        <v>0.8541666666666666</v>
       </c>
       <c r="E25" s="5">
-        <v>0.9895833333333334</v>
+        <v>0.8958333333333334</v>
       </c>
       <c r="F25" s="1" t="s">
         <v>198</v>
@@ -3993,19 +3996,19 @@
     </row>
     <row r="26">
       <c r="A26" s="1" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="B26" s="1" t="s">
         <v>28</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>48</v>
+        <v>29</v>
       </c>
       <c r="D26" s="5">
-        <v>0.5416666666666666</v>
+        <v>0.8958333333333334</v>
       </c>
       <c r="E26" s="5">
-        <v>0.5833333333333334</v>
+        <v>0.9375</v>
       </c>
       <c r="F26" s="1" t="s">
         <v>198</v>
@@ -4013,19 +4016,19 @@
     </row>
     <row r="27">
       <c r="A27" s="1" t="s">
-        <v>205</v>
+        <v>47</v>
       </c>
       <c r="B27" s="1" t="s">
         <v>28</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>48</v>
+        <v>29</v>
       </c>
       <c r="D27" s="5">
-        <v>0.5833333333333334</v>
+        <v>0.9375</v>
       </c>
       <c r="E27" s="5">
-        <v>0.625</v>
+        <v>0.9895833333333334</v>
       </c>
       <c r="F27" s="1" t="s">
         <v>198</v>
@@ -4033,7 +4036,7 @@
     </row>
     <row r="28">
       <c r="A28" s="1" t="s">
-        <v>31</v>
+        <v>49</v>
       </c>
       <c r="B28" s="1" t="s">
         <v>28</v>
@@ -4042,10 +4045,10 @@
         <v>48</v>
       </c>
       <c r="D28" s="5">
-        <v>0.625</v>
+        <v>0.5416666666666666</v>
       </c>
       <c r="E28" s="5">
-        <v>0.6666666666666666</v>
+        <v>0.5833333333333334</v>
       </c>
       <c r="F28" s="1" t="s">
         <v>198</v>
@@ -4053,7 +4056,7 @@
     </row>
     <row r="29">
       <c r="A29" s="1" t="s">
-        <v>52</v>
+        <v>205</v>
       </c>
       <c r="B29" s="1" t="s">
         <v>28</v>
@@ -4062,10 +4065,10 @@
         <v>48</v>
       </c>
       <c r="D29" s="5">
-        <v>0.6666666666666666</v>
+        <v>0.5833333333333334</v>
       </c>
       <c r="E29" s="5">
-        <v>0.7291666666666666</v>
+        <v>0.625</v>
       </c>
       <c r="F29" s="1" t="s">
         <v>198</v>
@@ -4073,7 +4076,7 @@
     </row>
     <row r="30">
       <c r="A30" s="1" t="s">
-        <v>55</v>
+        <v>31</v>
       </c>
       <c r="B30" s="1" t="s">
         <v>28</v>
@@ -4082,10 +4085,10 @@
         <v>48</v>
       </c>
       <c r="D30" s="5">
-        <v>0.7291666666666666</v>
+        <v>0.625</v>
       </c>
       <c r="E30" s="5">
-        <v>0.7916666666666666</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="F30" s="1" t="s">
         <v>198</v>
@@ -4093,7 +4096,7 @@
     </row>
     <row r="31">
       <c r="A31" s="1" t="s">
-        <v>206</v>
+        <v>52</v>
       </c>
       <c r="B31" s="1" t="s">
         <v>28</v>
@@ -4102,10 +4105,10 @@
         <v>48</v>
       </c>
       <c r="D31" s="5">
-        <v>0.7916666666666666</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="E31" s="5">
-        <v>0.8541666666666666</v>
+        <v>0.7291666666666666</v>
       </c>
       <c r="F31" s="1" t="s">
         <v>198</v>
@@ -4113,7 +4116,7 @@
     </row>
     <row r="32">
       <c r="A32" s="1" t="s">
-        <v>207</v>
+        <v>55</v>
       </c>
       <c r="B32" s="1" t="s">
         <v>28</v>
@@ -4122,10 +4125,10 @@
         <v>48</v>
       </c>
       <c r="D32" s="5">
-        <v>0.8541666666666666</v>
+        <v>0.7291666666666666</v>
       </c>
       <c r="E32" s="5">
-        <v>0.9895833333333334</v>
+        <v>0.7916666666666666</v>
       </c>
       <c r="F32" s="1" t="s">
         <v>198</v>
@@ -4133,19 +4136,19 @@
     </row>
     <row r="33">
       <c r="A33" s="1" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B33" s="1" t="s">
         <v>28</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>63</v>
+        <v>48</v>
       </c>
       <c r="D33" s="5">
-        <v>0.5416666666666666</v>
+        <v>0.7916666666666666</v>
       </c>
       <c r="E33" s="5">
-        <v>0.5625</v>
+        <v>0.8541666666666666</v>
       </c>
       <c r="F33" s="1" t="s">
         <v>198</v>
@@ -4153,19 +4156,19 @@
     </row>
     <row r="34">
       <c r="A34" s="1" t="s">
-        <v>67</v>
+        <v>208</v>
       </c>
       <c r="B34" s="1" t="s">
         <v>28</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>63</v>
+        <v>48</v>
       </c>
       <c r="D34" s="5">
-        <v>0.5625</v>
+        <v>0.8541666666666666</v>
       </c>
       <c r="E34" s="5">
-        <v>0.59375</v>
+        <v>0.9895833333333334</v>
       </c>
       <c r="F34" s="1" t="s">
         <v>198</v>
@@ -4173,7 +4176,7 @@
     </row>
     <row r="35">
       <c r="A35" s="1" t="s">
-        <v>69</v>
+        <v>209</v>
       </c>
       <c r="B35" s="1" t="s">
         <v>28</v>
@@ -4182,10 +4185,10 @@
         <v>63</v>
       </c>
       <c r="D35" s="5">
-        <v>0.59375</v>
+        <v>0.5416666666666666</v>
       </c>
       <c r="E35" s="5">
-        <v>0.75</v>
+        <v>0.5625</v>
       </c>
       <c r="F35" s="1" t="s">
         <v>198</v>
@@ -4193,7 +4196,7 @@
     </row>
     <row r="36">
       <c r="A36" s="1" t="s">
-        <v>209</v>
+        <v>67</v>
       </c>
       <c r="B36" s="1" t="s">
         <v>28</v>
@@ -4202,10 +4205,10 @@
         <v>63</v>
       </c>
       <c r="D36" s="5">
-        <v>0.75</v>
+        <v>0.5625</v>
       </c>
       <c r="E36" s="5">
-        <v>0.7916666666666666</v>
+        <v>0.59375</v>
       </c>
       <c r="F36" s="1" t="s">
         <v>198</v>
@@ -4213,199 +4216,199 @@
     </row>
     <row r="37">
       <c r="A37" s="1" t="s">
-        <v>86</v>
+        <v>69</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>210</v>
+        <v>28</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>29</v>
+        <v>63</v>
       </c>
       <c r="D37" s="5">
-        <v>0.625</v>
+        <v>0.59375</v>
       </c>
       <c r="E37" s="5">
-        <v>0.6875</v>
+        <v>0.75</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>211</v>
+        <v>198</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="s">
-        <v>88</v>
+        <v>210</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>210</v>
+        <v>28</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>29</v>
+        <v>63</v>
       </c>
       <c r="D38" s="5">
-        <v>0.6875</v>
+        <v>0.75</v>
       </c>
       <c r="E38" s="5">
-        <v>0.7395833333333334</v>
+        <v>0.7916666666666666</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>211</v>
+        <v>198</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="C39" s="1" t="s">
         <v>29</v>
       </c>
       <c r="D39" s="5">
-        <v>0.7395833333333334</v>
+        <v>0.625</v>
       </c>
       <c r="E39" s="5">
-        <v>0.7916666666666666</v>
+        <v>0.6875</v>
       </c>
       <c r="F39" s="1" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="C40" s="1" t="s">
         <v>29</v>
       </c>
       <c r="D40" s="5">
-        <v>0.7916666666666666</v>
+        <v>0.6875</v>
       </c>
       <c r="E40" s="5">
-        <v>0.8541666666666666</v>
+        <v>0.7395833333333334</v>
       </c>
       <c r="F40" s="1" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="C41" s="1" t="s">
         <v>29</v>
       </c>
       <c r="D41" s="5">
-        <v>0.8541666666666666</v>
+        <v>0.7395833333333334</v>
       </c>
       <c r="E41" s="5">
-        <v>0.9166666666666666</v>
+        <v>0.7916666666666666</v>
       </c>
       <c r="F41" s="1" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="C42" s="1" t="s">
         <v>29</v>
       </c>
       <c r="D42" s="5">
-        <v>0.9166666666666666</v>
+        <v>0.7916666666666666</v>
       </c>
       <c r="E42" s="5">
-        <v>0.9791666666666666</v>
+        <v>0.8541666666666666</v>
       </c>
       <c r="F42" s="1" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="B43" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="C43" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="D43" s="5">
+        <v>0.8541666666666666</v>
+      </c>
+      <c r="E43" s="5">
+        <v>0.9166666666666666</v>
+      </c>
+      <c r="F43" s="1" t="s">
         <v>212</v>
-      </c>
-      <c r="C43" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="D43" s="5">
-        <v>0.5</v>
-      </c>
-      <c r="E43" s="5">
-        <v>0.5520833333333334</v>
-      </c>
-      <c r="F43" s="1" t="s">
-        <v>211</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="B44" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="C44" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="D44" s="5">
+        <v>0.9166666666666666</v>
+      </c>
+      <c r="E44" s="5">
+        <v>0.9791666666666666</v>
+      </c>
+      <c r="F44" s="1" t="s">
         <v>212</v>
-      </c>
-      <c r="C44" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="D44" s="5">
-        <v>0.5520833333333334</v>
-      </c>
-      <c r="E44" s="5">
-        <v>0.6041666666666666</v>
-      </c>
-      <c r="F44" s="1" t="s">
-        <v>198</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="B45" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="C45" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D45" s="5">
+        <v>0.5</v>
+      </c>
+      <c r="E45" s="5">
+        <v>0.5520833333333334</v>
+      </c>
+      <c r="F45" s="1" t="s">
         <v>212</v>
-      </c>
-      <c r="C45" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="D45" s="5">
-        <v>0.6041666666666666</v>
-      </c>
-      <c r="E45" s="5">
-        <v>0.65625</v>
-      </c>
-      <c r="F45" s="1" t="s">
-        <v>198</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="C46" s="1" t="s">
         <v>48</v>
       </c>
       <c r="D46" s="5">
-        <v>0.65625</v>
+        <v>0.5520833333333334</v>
       </c>
       <c r="E46" s="5">
-        <v>0.7083333333333334</v>
+        <v>0.6041666666666666</v>
       </c>
       <c r="F46" s="1" t="s">
         <v>198</v>
@@ -4413,19 +4416,19 @@
     </row>
     <row r="47">
       <c r="A47" s="1" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="C47" s="1" t="s">
         <v>48</v>
       </c>
       <c r="D47" s="5">
-        <v>0.7083333333333334</v>
+        <v>0.6041666666666666</v>
       </c>
       <c r="E47" s="5">
-        <v>0.7604166666666666</v>
+        <v>0.65625</v>
       </c>
       <c r="F47" s="1" t="s">
         <v>198</v>
@@ -4433,19 +4436,19 @@
     </row>
     <row r="48">
       <c r="A48" s="1" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="C48" s="1" t="s">
         <v>48</v>
       </c>
       <c r="D48" s="5">
-        <v>0.7604166666666666</v>
+        <v>0.65625</v>
       </c>
       <c r="E48" s="5">
-        <v>0.8125</v>
+        <v>0.7083333333333334</v>
       </c>
       <c r="F48" s="1" t="s">
         <v>198</v>
@@ -4453,19 +4456,19 @@
     </row>
     <row r="49">
       <c r="A49" s="1" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="C49" s="1" t="s">
         <v>48</v>
       </c>
       <c r="D49" s="5">
-        <v>0.8125</v>
+        <v>0.7083333333333334</v>
       </c>
       <c r="E49" s="5">
-        <v>0.84375</v>
+        <v>0.7604166666666666</v>
       </c>
       <c r="F49" s="1" t="s">
         <v>198</v>
@@ -4473,19 +4476,19 @@
     </row>
     <row r="50">
       <c r="A50" s="1" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="C50" s="1" t="s">
         <v>48</v>
       </c>
       <c r="D50" s="5">
-        <v>0.84375</v>
+        <v>0.7604166666666666</v>
       </c>
       <c r="E50" s="5">
-        <v>0.8958333333333334</v>
+        <v>0.8125</v>
       </c>
       <c r="F50" s="1" t="s">
         <v>198</v>
@@ -4493,19 +4496,19 @@
     </row>
     <row r="51">
       <c r="A51" s="1" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="C51" s="1" t="s">
         <v>48</v>
       </c>
       <c r="D51" s="5">
-        <v>0.8958333333333334</v>
+        <v>0.8125</v>
       </c>
       <c r="E51" s="5">
-        <v>0.9479166666666666</v>
+        <v>0.84375</v>
       </c>
       <c r="F51" s="1" t="s">
         <v>198</v>
@@ -4513,19 +4516,19 @@
     </row>
     <row r="52">
       <c r="A52" s="1" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="C52" s="1" t="s">
         <v>48</v>
       </c>
       <c r="D52" s="5">
-        <v>0.9479166666666666</v>
+        <v>0.84375</v>
       </c>
       <c r="E52" s="5">
-        <v>0.0</v>
+        <v>0.8958333333333334</v>
       </c>
       <c r="F52" s="1" t="s">
         <v>198</v>
@@ -4533,139 +4536,139 @@
     </row>
     <row r="53">
       <c r="A53" s="1" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>63</v>
+        <v>48</v>
       </c>
       <c r="D53" s="5">
-        <v>0.5</v>
+        <v>0.8958333333333334</v>
       </c>
       <c r="E53" s="5">
-        <v>0.5833333333333334</v>
+        <v>0.9479166666666666</v>
       </c>
       <c r="F53" s="1" t="s">
-        <v>211</v>
+        <v>198</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="1" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>63</v>
+        <v>48</v>
       </c>
       <c r="D54" s="5">
-        <v>0.5833333333333334</v>
+        <v>0.9479166666666666</v>
       </c>
       <c r="E54" s="5">
-        <v>0.6354166666666666</v>
+        <v>0.0</v>
       </c>
       <c r="F54" s="1" t="s">
-        <v>211</v>
+        <v>198</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="1" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="C55" s="1" t="s">
         <v>63</v>
       </c>
       <c r="D55" s="5">
-        <v>0.6354166666666666</v>
+        <v>0.5</v>
       </c>
       <c r="E55" s="5">
-        <v>0.7083333333333334</v>
+        <v>0.5833333333333334</v>
       </c>
       <c r="F55" s="1" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="1" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="C56" s="1" t="s">
         <v>63</v>
       </c>
       <c r="D56" s="5">
-        <v>0.7083333333333334</v>
+        <v>0.5833333333333334</v>
       </c>
       <c r="E56" s="5">
-        <v>0.7916666666666666</v>
+        <v>0.6354166666666666</v>
       </c>
       <c r="F56" s="1" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="1" t="s">
-        <v>213</v>
+        <v>124</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>29</v>
+        <v>63</v>
       </c>
       <c r="D57" s="5">
-        <v>0.6145833333333334</v>
+        <v>0.6354166666666666</v>
       </c>
       <c r="E57" s="5">
-        <v>0.6666666666666666</v>
+        <v>0.7083333333333334</v>
       </c>
       <c r="F57" s="1" t="s">
-        <v>198</v>
+        <v>212</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="1" t="s">
-        <v>133</v>
+        <v>126</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>29</v>
+        <v>63</v>
       </c>
       <c r="D58" s="5">
-        <v>0.6666666666666666</v>
+        <v>0.7083333333333334</v>
       </c>
       <c r="E58" s="5">
-        <v>0.71875</v>
+        <v>0.7916666666666666</v>
       </c>
       <c r="F58" s="1" t="s">
-        <v>198</v>
+        <v>212</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="1" t="s">
-        <v>79</v>
+        <v>214</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C59" s="1" t="s">
         <v>29</v>
       </c>
       <c r="D59" s="5">
-        <v>0.71875</v>
+        <v>0.6145833333333334</v>
       </c>
       <c r="E59" s="5">
-        <v>0.7708333333333334</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="F59" s="1" t="s">
         <v>198</v>
@@ -4673,19 +4676,19 @@
     </row>
     <row r="60">
       <c r="A60" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="B60" s="1" t="s">
         <v>215</v>
       </c>
-      <c r="B60" s="1" t="s">
-        <v>214</v>
-      </c>
       <c r="C60" s="1" t="s">
         <v>29</v>
       </c>
       <c r="D60" s="5">
-        <v>0.7708333333333334</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="E60" s="5">
-        <v>0.8229166666666666</v>
+        <v>0.71875</v>
       </c>
       <c r="F60" s="1" t="s">
         <v>198</v>
@@ -4693,19 +4696,19 @@
     </row>
     <row r="61">
       <c r="A61" s="1" t="s">
-        <v>114</v>
+        <v>79</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C61" s="1" t="s">
         <v>29</v>
       </c>
       <c r="D61" s="5">
-        <v>0.8229166666666666</v>
+        <v>0.71875</v>
       </c>
       <c r="E61" s="5">
-        <v>0.875</v>
+        <v>0.7708333333333334</v>
       </c>
       <c r="F61" s="1" t="s">
         <v>198</v>
@@ -4713,19 +4716,19 @@
     </row>
     <row r="62">
       <c r="A62" s="1" t="s">
-        <v>108</v>
+        <v>216</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C62" s="1" t="s">
         <v>29</v>
       </c>
       <c r="D62" s="5">
-        <v>0.875</v>
+        <v>0.7708333333333334</v>
       </c>
       <c r="E62" s="5">
-        <v>0.9270833333333334</v>
+        <v>0.8229166666666666</v>
       </c>
       <c r="F62" s="1" t="s">
         <v>198</v>
@@ -4733,19 +4736,19 @@
     </row>
     <row r="63">
       <c r="A63" s="1" t="s">
-        <v>214</v>
+        <v>114</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C63" s="1" t="s">
         <v>29</v>
       </c>
       <c r="D63" s="5">
-        <v>0.9270833333333334</v>
+        <v>0.8229166666666666</v>
       </c>
       <c r="E63" s="5">
-        <v>0.9895833333333334</v>
+        <v>0.875</v>
       </c>
       <c r="F63" s="1" t="s">
         <v>198</v>
@@ -4753,19 +4756,19 @@
     </row>
     <row r="64">
       <c r="A64" s="1" t="s">
-        <v>216</v>
+        <v>108</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>48</v>
+        <v>29</v>
       </c>
       <c r="D64" s="5">
-        <v>0.53125</v>
+        <v>0.875</v>
       </c>
       <c r="E64" s="5">
-        <v>0.5833333333333334</v>
+        <v>0.9270833333333334</v>
       </c>
       <c r="F64" s="1" t="s">
         <v>198</v>
@@ -4773,19 +4776,19 @@
     </row>
     <row r="65">
       <c r="A65" s="1" t="s">
-        <v>133</v>
+        <v>215</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C65" s="1" t="s">
-        <v>48</v>
+        <v>29</v>
       </c>
       <c r="D65" s="5">
-        <v>0.5833333333333334</v>
+        <v>0.9270833333333334</v>
       </c>
       <c r="E65" s="5">
-        <v>0.6354166666666666</v>
+        <v>0.9895833333333334</v>
       </c>
       <c r="F65" s="1" t="s">
         <v>198</v>
@@ -4796,16 +4799,16 @@
         <v>217</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C66" s="1" t="s">
         <v>48</v>
       </c>
       <c r="D66" s="5">
-        <v>0.6354166666666666</v>
+        <v>0.53125</v>
       </c>
       <c r="E66" s="5">
-        <v>0.6875</v>
+        <v>0.5833333333333334</v>
       </c>
       <c r="F66" s="1" t="s">
         <v>198</v>
@@ -4813,19 +4816,19 @@
     </row>
     <row r="67">
       <c r="A67" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="B67" s="1" t="s">
         <v>215</v>
       </c>
-      <c r="B67" s="1" t="s">
-        <v>214</v>
-      </c>
       <c r="C67" s="1" t="s">
         <v>48</v>
       </c>
       <c r="D67" s="5">
-        <v>0.6875</v>
+        <v>0.5833333333333334</v>
       </c>
       <c r="E67" s="5">
-        <v>0.7395833333333334</v>
+        <v>0.6354166666666666</v>
       </c>
       <c r="F67" s="1" t="s">
         <v>198</v>
@@ -4833,19 +4836,19 @@
     </row>
     <row r="68">
       <c r="A68" s="1" t="s">
-        <v>129</v>
+        <v>218</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C68" s="1" t="s">
         <v>48</v>
       </c>
       <c r="D68" s="5">
-        <v>0.7395833333333334</v>
+        <v>0.6354166666666666</v>
       </c>
       <c r="E68" s="5">
-        <v>0.78125</v>
+        <v>0.6875</v>
       </c>
       <c r="F68" s="1" t="s">
         <v>198</v>
@@ -4853,19 +4856,19 @@
     </row>
     <row r="69">
       <c r="A69" s="1" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C69" s="1" t="s">
         <v>48</v>
       </c>
       <c r="D69" s="5">
-        <v>0.78125</v>
+        <v>0.6875</v>
       </c>
       <c r="E69" s="5">
-        <v>0.8333333333333334</v>
+        <v>0.7395833333333334</v>
       </c>
       <c r="F69" s="1" t="s">
         <v>198</v>
@@ -4873,19 +4876,19 @@
     </row>
     <row r="70">
       <c r="A70" s="1" t="s">
-        <v>139</v>
+        <v>129</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C70" s="1" t="s">
         <v>48</v>
       </c>
       <c r="D70" s="5">
-        <v>0.8333333333333334</v>
+        <v>0.7395833333333334</v>
       </c>
       <c r="E70" s="5">
-        <v>0.9166666666666666</v>
+        <v>0.78125</v>
       </c>
       <c r="F70" s="1" t="s">
         <v>198</v>
@@ -4896,16 +4899,16 @@
         <v>219</v>
       </c>
       <c r="B71" s="1" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C71" s="1" t="s">
         <v>48</v>
       </c>
       <c r="D71" s="5">
-        <v>0.9166666666666666</v>
+        <v>0.78125</v>
       </c>
       <c r="E71" s="5">
-        <v>0.0</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="F71" s="1" t="s">
         <v>198</v>
@@ -4913,19 +4916,19 @@
     </row>
     <row r="72">
       <c r="A72" s="1" t="s">
-        <v>220</v>
+        <v>139</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>221</v>
+        <v>215</v>
       </c>
       <c r="C72" s="1" t="s">
-        <v>63</v>
+        <v>48</v>
       </c>
       <c r="D72" s="5">
-        <v>0.5</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="E72" s="5">
-        <v>0.7916666666666666</v>
+        <v>0.9166666666666666</v>
       </c>
       <c r="F72" s="1" t="s">
         <v>198</v>
@@ -4933,239 +4936,239 @@
     </row>
     <row r="73">
       <c r="A73" s="1" t="s">
-        <v>142</v>
+        <v>220</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>222</v>
+        <v>215</v>
       </c>
       <c r="C73" s="1" t="s">
-        <v>29</v>
+        <v>48</v>
       </c>
       <c r="D73" s="5">
-        <v>0.6458333333333334</v>
+        <v>0.9166666666666666</v>
       </c>
       <c r="E73" s="5">
-        <v>0.6979166666666666</v>
+        <v>0.0</v>
       </c>
       <c r="F73" s="1" t="s">
-        <v>223</v>
+        <v>198</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="1" t="s">
-        <v>145</v>
+        <v>221</v>
       </c>
       <c r="B74" s="1" t="s">
         <v>222</v>
       </c>
       <c r="C74" s="1" t="s">
-        <v>29</v>
+        <v>63</v>
       </c>
       <c r="D74" s="5">
-        <v>0.71875</v>
+        <v>0.5</v>
       </c>
       <c r="E74" s="5">
-        <v>0.7708333333333334</v>
+        <v>0.7916666666666666</v>
       </c>
       <c r="F74" s="1" t="s">
-        <v>223</v>
+        <v>198</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="1" t="s">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="B75" s="1" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="C75" s="1" t="s">
         <v>29</v>
       </c>
       <c r="D75" s="5">
-        <v>0.7916666666666666</v>
+        <v>0.6458333333333334</v>
       </c>
       <c r="E75" s="5">
-        <v>0.84375</v>
+        <v>0.6979166666666666</v>
       </c>
       <c r="F75" s="1" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="1" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="B76" s="1" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="C76" s="1" t="s">
         <v>29</v>
       </c>
       <c r="D76" s="5">
-        <v>0.8645833333333334</v>
+        <v>0.71875</v>
       </c>
       <c r="E76" s="5">
-        <v>0.9166666666666666</v>
+        <v>0.7708333333333334</v>
       </c>
       <c r="F76" s="1" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="1" t="s">
-        <v>155</v>
+        <v>148</v>
       </c>
       <c r="B77" s="1" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="C77" s="1" t="s">
         <v>29</v>
       </c>
       <c r="D77" s="5">
-        <v>0.9270833333333334</v>
+        <v>0.7916666666666666</v>
       </c>
       <c r="E77" s="5">
-        <v>0.9895833333333334</v>
+        <v>0.84375</v>
       </c>
       <c r="F77" s="1" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="1" t="s">
-        <v>157</v>
+        <v>151</v>
       </c>
       <c r="B78" s="1" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="C78" s="1" t="s">
-        <v>48</v>
+        <v>29</v>
       </c>
       <c r="D78" s="5">
-        <v>0.5625</v>
+        <v>0.8645833333333334</v>
       </c>
       <c r="E78" s="5">
-        <v>0.6145833333333334</v>
+        <v>0.9166666666666666</v>
       </c>
       <c r="F78" s="1" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="1" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="B79" s="1" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="C79" s="1" t="s">
-        <v>48</v>
+        <v>29</v>
       </c>
       <c r="D79" s="5">
-        <v>0.6354166666666666</v>
+        <v>0.9270833333333334</v>
       </c>
       <c r="E79" s="5">
-        <v>0.6875</v>
+        <v>0.9895833333333334</v>
       </c>
       <c r="F79" s="1" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="1" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="B80" s="1" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="C80" s="1" t="s">
         <v>48</v>
       </c>
       <c r="D80" s="5">
-        <v>0.7083333333333334</v>
+        <v>0.5625</v>
       </c>
       <c r="E80" s="5">
-        <v>0.7604166666666666</v>
+        <v>0.6145833333333334</v>
       </c>
       <c r="F80" s="1" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="1" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="B81" s="1" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="C81" s="1" t="s">
         <v>48</v>
       </c>
       <c r="D81" s="5">
-        <v>0.78125</v>
+        <v>0.6354166666666666</v>
       </c>
       <c r="E81" s="5">
-        <v>0.8229166666666666</v>
+        <v>0.6875</v>
       </c>
       <c r="F81" s="1" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="1" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="B82" s="1" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="C82" s="1" t="s">
         <v>48</v>
       </c>
       <c r="D82" s="5">
-        <v>0.84375</v>
+        <v>0.7083333333333334</v>
       </c>
       <c r="E82" s="5">
-        <v>0.8958333333333334</v>
+        <v>0.7604166666666666</v>
       </c>
       <c r="F82" s="1" t="s">
-        <v>198</v>
+        <v>224</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="1" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="B83" s="1" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="C83" s="1" t="s">
         <v>48</v>
       </c>
       <c r="D83" s="5">
-        <v>0.8958333333333334</v>
+        <v>0.78125</v>
       </c>
       <c r="E83" s="5">
-        <v>0.9791666666666666</v>
+        <v>0.8229166666666666</v>
       </c>
       <c r="F83" s="1" t="s">
-        <v>198</v>
+        <v>224</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="1" t="s">
-        <v>79</v>
+        <v>163</v>
       </c>
       <c r="B84" s="1" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="C84" s="1" t="s">
         <v>48</v>
       </c>
       <c r="D84" s="5">
-        <v>0.9791666666666666</v>
+        <v>0.84375</v>
       </c>
       <c r="E84" s="5">
-        <v>0.0</v>
+        <v>0.8958333333333334</v>
       </c>
       <c r="F84" s="1" t="s">
         <v>198</v>
@@ -5173,359 +5176,359 @@
     </row>
     <row r="85">
       <c r="A85" s="1" t="s">
-        <v>213</v>
+        <v>165</v>
       </c>
       <c r="B85" s="1" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C85" s="1" t="s">
-        <v>29</v>
+        <v>48</v>
       </c>
       <c r="D85" s="5">
-        <v>0.6354166666666666</v>
+        <v>0.8958333333333334</v>
       </c>
       <c r="E85" s="5">
-        <v>0.65625</v>
+        <v>0.9791666666666666</v>
       </c>
       <c r="F85" s="1" t="s">
-        <v>223</v>
+        <v>198</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="1" t="s">
-        <v>146</v>
+        <v>79</v>
       </c>
       <c r="B86" s="1" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C86" s="1" t="s">
-        <v>29</v>
+        <v>48</v>
       </c>
       <c r="D86" s="5">
-        <v>0.6770833333333334</v>
+        <v>0.9791666666666666</v>
       </c>
       <c r="E86" s="5">
-        <v>0.7395833333333334</v>
+        <v>0.0</v>
       </c>
       <c r="F86" s="1" t="s">
-        <v>223</v>
+        <v>198</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="1" t="s">
-        <v>174</v>
+        <v>214</v>
       </c>
       <c r="B87" s="1" t="s">
+        <v>225</v>
+      </c>
+      <c r="C87" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="D87" s="5">
+        <v>0.6354166666666666</v>
+      </c>
+      <c r="E87" s="5">
+        <v>0.65625</v>
+      </c>
+      <c r="F87" s="1" t="s">
         <v>224</v>
-      </c>
-      <c r="C87" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="D87" s="5">
-        <v>0.7604166666666666</v>
-      </c>
-      <c r="E87" s="5">
-        <v>0.8229166666666666</v>
-      </c>
-      <c r="F87" s="1" t="s">
-        <v>223</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="1" t="s">
-        <v>176</v>
+        <v>146</v>
       </c>
       <c r="B88" s="1" t="s">
+        <v>225</v>
+      </c>
+      <c r="C88" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="D88" s="5">
+        <v>0.6770833333333334</v>
+      </c>
+      <c r="E88" s="5">
+        <v>0.7395833333333334</v>
+      </c>
+      <c r="F88" s="1" t="s">
         <v>224</v>
-      </c>
-      <c r="C88" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="D88" s="5">
-        <v>0.84375</v>
-      </c>
-      <c r="E88" s="5">
-        <v>0.90625</v>
-      </c>
-      <c r="F88" s="1" t="s">
-        <v>223</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="1" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="B89" s="1" t="s">
+        <v>225</v>
+      </c>
+      <c r="C89" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="D89" s="5">
+        <v>0.7604166666666666</v>
+      </c>
+      <c r="E89" s="5">
+        <v>0.8229166666666666</v>
+      </c>
+      <c r="F89" s="1" t="s">
         <v>224</v>
-      </c>
-      <c r="C89" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="D89" s="5">
-        <v>0.9270833333333334</v>
-      </c>
-      <c r="E89" s="5">
-        <v>0.9895833333333334</v>
-      </c>
-      <c r="F89" s="1" t="s">
-        <v>223</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="1" t="s">
-        <v>169</v>
+        <v>176</v>
       </c>
       <c r="B90" s="1" t="s">
+        <v>225</v>
+      </c>
+      <c r="C90" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="D90" s="5">
+        <v>0.84375</v>
+      </c>
+      <c r="E90" s="5">
+        <v>0.90625</v>
+      </c>
+      <c r="F90" s="1" t="s">
         <v>224</v>
-      </c>
-      <c r="C90" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="D90" s="5">
-        <v>0.5520833333333334</v>
-      </c>
-      <c r="E90" s="5">
-        <v>0.59375</v>
-      </c>
-      <c r="F90" s="1" t="s">
-        <v>223</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="1" t="s">
-        <v>149</v>
+        <v>177</v>
       </c>
       <c r="B91" s="1" t="s">
+        <v>225</v>
+      </c>
+      <c r="C91" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="D91" s="5">
+        <v>0.9270833333333334</v>
+      </c>
+      <c r="E91" s="5">
+        <v>0.9895833333333334</v>
+      </c>
+      <c r="F91" s="1" t="s">
         <v>224</v>
-      </c>
-      <c r="C91" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="D91" s="5">
-        <v>0.6145833333333334</v>
-      </c>
-      <c r="E91" s="5">
-        <v>0.6770833333333334</v>
-      </c>
-      <c r="F91" s="1" t="s">
-        <v>223</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="1" t="s">
-        <v>182</v>
+        <v>169</v>
       </c>
       <c r="B92" s="1" t="s">
+        <v>225</v>
+      </c>
+      <c r="C92" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D92" s="5">
+        <v>0.5520833333333334</v>
+      </c>
+      <c r="E92" s="5">
+        <v>0.59375</v>
+      </c>
+      <c r="F92" s="1" t="s">
         <v>224</v>
-      </c>
-      <c r="C92" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="D92" s="5">
-        <v>0.6979166666666666</v>
-      </c>
-      <c r="E92" s="5">
-        <v>0.7604166666666666</v>
-      </c>
-      <c r="F92" s="1" t="s">
-        <v>223</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="1" t="s">
-        <v>184</v>
+        <v>149</v>
       </c>
       <c r="B93" s="1" t="s">
+        <v>225</v>
+      </c>
+      <c r="C93" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D93" s="5">
+        <v>0.6145833333333334</v>
+      </c>
+      <c r="E93" s="5">
+        <v>0.6770833333333334</v>
+      </c>
+      <c r="F93" s="1" t="s">
         <v>224</v>
-      </c>
-      <c r="C93" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="D93" s="5">
-        <v>0.78125</v>
-      </c>
-      <c r="E93" s="5">
-        <v>0.84375</v>
-      </c>
-      <c r="F93" s="1" t="s">
-        <v>223</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="1" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="B94" s="1" t="s">
+        <v>225</v>
+      </c>
+      <c r="C94" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D94" s="5">
+        <v>0.6979166666666666</v>
+      </c>
+      <c r="E94" s="5">
+        <v>0.7604166666666666</v>
+      </c>
+      <c r="F94" s="1" t="s">
         <v>224</v>
-      </c>
-      <c r="C94" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="D94" s="5">
-        <v>0.8645833333333334</v>
-      </c>
-      <c r="E94" s="5">
-        <v>0.9270833333333334</v>
-      </c>
-      <c r="F94" s="1" t="s">
-        <v>223</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="1" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="B95" s="1" t="s">
+        <v>225</v>
+      </c>
+      <c r="C95" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D95" s="5">
+        <v>0.78125</v>
+      </c>
+      <c r="E95" s="5">
+        <v>0.84375</v>
+      </c>
+      <c r="F95" s="1" t="s">
         <v>224</v>
-      </c>
-      <c r="C95" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="D95" s="5">
-        <v>0.9479166666666666</v>
-      </c>
-      <c r="E95" s="5">
-        <v>0.0</v>
-      </c>
-      <c r="F95" s="1" t="s">
-        <v>223</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="1" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="B96" s="1" t="s">
+        <v>225</v>
+      </c>
+      <c r="C96" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D96" s="5">
+        <v>0.8645833333333334</v>
+      </c>
+      <c r="E96" s="5">
+        <v>0.9270833333333334</v>
+      </c>
+      <c r="F96" s="1" t="s">
         <v>224</v>
-      </c>
-      <c r="C96" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="D96" s="5">
-        <v>0.5625</v>
-      </c>
-      <c r="E96" s="5">
-        <v>0.6145833333333334</v>
-      </c>
-      <c r="F96" s="1" t="s">
-        <v>223</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="1" t="s">
-        <v>153</v>
+        <v>187</v>
       </c>
       <c r="B97" s="1" t="s">
+        <v>225</v>
+      </c>
+      <c r="C97" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D97" s="5">
+        <v>0.9479166666666666</v>
+      </c>
+      <c r="E97" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="F97" s="1" t="s">
         <v>224</v>
-      </c>
-      <c r="C97" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="D97" s="5">
-        <v>0.6354166666666666</v>
-      </c>
-      <c r="E97" s="5">
-        <v>0.6875</v>
-      </c>
-      <c r="F97" s="1" t="s">
-        <v>223</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="1" t="s">
-        <v>148</v>
+        <v>188</v>
       </c>
       <c r="B98" s="1" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="C98" s="1" t="s">
         <v>63</v>
       </c>
       <c r="D98" s="5">
-        <v>0.7083333333333334</v>
+        <v>0.5625</v>
       </c>
       <c r="E98" s="5">
-        <v>0.7604166666666666</v>
+        <v>0.6145833333333334</v>
       </c>
       <c r="F98" s="1" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="1" t="s">
-        <v>160</v>
+        <v>153</v>
       </c>
       <c r="B99" s="1" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="C99" s="1" t="s">
         <v>63</v>
       </c>
       <c r="D99" s="5">
-        <v>0.78125</v>
+        <v>0.6354166666666666</v>
       </c>
       <c r="E99" s="5">
-        <v>0.8333333333333334</v>
+        <v>0.6875</v>
       </c>
       <c r="F99" s="1" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="B100" s="1" t="s">
         <v>225</v>
-      </c>
-      <c r="B100" s="1" t="s">
-        <v>224</v>
       </c>
       <c r="C100" s="1" t="s">
         <v>63</v>
       </c>
       <c r="D100" s="5">
-        <v>0.8333333333333334</v>
+        <v>0.7083333333333334</v>
       </c>
       <c r="E100" s="5">
-        <v>0.9166666666666666</v>
+        <v>0.7604166666666666</v>
       </c>
       <c r="F100" s="1" t="s">
-        <v>198</v>
+        <v>224</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="1" t="s">
-        <v>226</v>
+        <v>160</v>
       </c>
       <c r="B101" s="1" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="C101" s="1" t="s">
-        <v>29</v>
+        <v>63</v>
       </c>
       <c r="D101" s="5">
-        <v>0.5833333333333334</v>
+        <v>0.78125</v>
       </c>
       <c r="E101" s="5">
-        <v>0.625</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="F101" s="1" t="s">
-        <v>198</v>
+        <v>224</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="1" t="s">
-        <v>80</v>
+        <v>226</v>
       </c>
       <c r="B102" s="1" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="C102" s="1" t="s">
-        <v>29</v>
+        <v>63</v>
       </c>
       <c r="D102" s="5">
-        <v>0.625</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="E102" s="5">
-        <v>0.6666666666666666</v>
+        <v>0.9166666666666666</v>
       </c>
       <c r="F102" s="1" t="s">
         <v>198</v>
@@ -5533,19 +5536,19 @@
     </row>
     <row r="103">
       <c r="A103" s="1" t="s">
+        <v>227</v>
+      </c>
+      <c r="B103" s="1" t="s">
         <v>228</v>
       </c>
-      <c r="B103" s="1" t="s">
-        <v>227</v>
-      </c>
       <c r="C103" s="1" t="s">
         <v>29</v>
       </c>
       <c r="D103" s="5">
-        <v>0.6666666666666666</v>
+        <v>0.5833333333333334</v>
       </c>
       <c r="E103" s="5">
-        <v>0.7291666666666666</v>
+        <v>0.625</v>
       </c>
       <c r="F103" s="1" t="s">
         <v>198</v>
@@ -5553,19 +5556,19 @@
     </row>
     <row r="104">
       <c r="A104" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B104" s="1" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="C104" s="1" t="s">
         <v>29</v>
       </c>
       <c r="D104" s="5">
-        <v>0.7291666666666666</v>
+        <v>0.625</v>
       </c>
       <c r="E104" s="5">
-        <v>0.7916666666666666</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="F104" s="1" t="s">
         <v>198</v>
@@ -5573,19 +5576,19 @@
     </row>
     <row r="105">
       <c r="A105" s="1" t="s">
-        <v>76</v>
+        <v>229</v>
       </c>
       <c r="B105" s="1" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="C105" s="1" t="s">
         <v>29</v>
       </c>
       <c r="D105" s="5">
-        <v>0.7916666666666666</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="E105" s="5">
-        <v>0.8541666666666666</v>
+        <v>0.7291666666666666</v>
       </c>
       <c r="F105" s="1" t="s">
         <v>198</v>
@@ -5593,19 +5596,19 @@
     </row>
     <row r="106">
       <c r="A106" s="1" t="s">
-        <v>73</v>
+        <v>81</v>
       </c>
       <c r="B106" s="1" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="C106" s="1" t="s">
         <v>29</v>
       </c>
       <c r="D106" s="5">
-        <v>0.8541666666666666</v>
+        <v>0.7291666666666666</v>
       </c>
       <c r="E106" s="5">
-        <v>0.90625</v>
+        <v>0.7916666666666666</v>
       </c>
       <c r="F106" s="1" t="s">
         <v>198</v>
@@ -5613,19 +5616,19 @@
     </row>
     <row r="107">
       <c r="A107" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B107" s="1" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="C107" s="1" t="s">
         <v>29</v>
       </c>
       <c r="D107" s="5">
-        <v>0.90625</v>
+        <v>0.7916666666666666</v>
       </c>
       <c r="E107" s="5">
-        <v>0.9895833333333334</v>
+        <v>0.8541666666666666</v>
       </c>
       <c r="F107" s="1" t="s">
         <v>198</v>
@@ -5636,16 +5639,16 @@
         <v>73</v>
       </c>
       <c r="B108" s="1" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="C108" s="1" t="s">
-        <v>48</v>
+        <v>29</v>
       </c>
       <c r="D108" s="5">
-        <v>0.5833333333333334</v>
+        <v>0.8541666666666666</v>
       </c>
       <c r="E108" s="5">
-        <v>0.6666666666666666</v>
+        <v>0.90625</v>
       </c>
       <c r="F108" s="1" t="s">
         <v>198</v>
@@ -5653,19 +5656,19 @@
     </row>
     <row r="109">
       <c r="A109" s="1" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="B109" s="1" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="C109" s="1" t="s">
-        <v>48</v>
+        <v>29</v>
       </c>
       <c r="D109" s="5">
-        <v>0.6666666666666666</v>
+        <v>0.90625</v>
       </c>
       <c r="E109" s="5">
-        <v>0.75</v>
+        <v>0.9895833333333334</v>
       </c>
       <c r="F109" s="1" t="s">
         <v>198</v>
@@ -5673,19 +5676,19 @@
     </row>
     <row r="110">
       <c r="A110" s="1" t="s">
-        <v>81</v>
+        <v>73</v>
       </c>
       <c r="B110" s="1" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="C110" s="1" t="s">
         <v>48</v>
       </c>
       <c r="D110" s="5">
-        <v>0.75</v>
+        <v>0.5833333333333334</v>
       </c>
       <c r="E110" s="5">
-        <v>0.8125</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="F110" s="1" t="s">
         <v>198</v>
@@ -5693,19 +5696,19 @@
     </row>
     <row r="111">
       <c r="A111" s="1" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="B111" s="1" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="C111" s="1" t="s">
         <v>48</v>
       </c>
       <c r="D111" s="5">
-        <v>0.8125</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="E111" s="5">
-        <v>0.8645833333333334</v>
+        <v>0.75</v>
       </c>
       <c r="F111" s="1" t="s">
         <v>198</v>
@@ -5713,19 +5716,19 @@
     </row>
     <row r="112">
       <c r="A112" s="1" t="s">
-        <v>229</v>
+        <v>81</v>
       </c>
       <c r="B112" s="1" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="C112" s="1" t="s">
         <v>48</v>
       </c>
       <c r="D112" s="5">
-        <v>0.8645833333333334</v>
+        <v>0.75</v>
       </c>
       <c r="E112" s="5">
-        <v>0.0</v>
+        <v>0.8125</v>
       </c>
       <c r="F112" s="1" t="s">
         <v>198</v>
@@ -5736,16 +5739,16 @@
         <v>78</v>
       </c>
       <c r="B113" s="1" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="C113" s="1" t="s">
-        <v>63</v>
+        <v>48</v>
       </c>
       <c r="D113" s="5">
-        <v>0.5</v>
+        <v>0.8125</v>
       </c>
       <c r="E113" s="5">
-        <v>0.5833333333333334</v>
+        <v>0.8645833333333334</v>
       </c>
       <c r="F113" s="1" t="s">
         <v>198</v>
@@ -5753,19 +5756,19 @@
     </row>
     <row r="114">
       <c r="A114" s="1" t="s">
-        <v>82</v>
+        <v>230</v>
       </c>
       <c r="B114" s="1" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="C114" s="1" t="s">
-        <v>63</v>
+        <v>48</v>
       </c>
       <c r="D114" s="5">
-        <v>0.5833333333333334</v>
+        <v>0.8645833333333334</v>
       </c>
       <c r="E114" s="5">
-        <v>0.6666666666666666</v>
+        <v>0.0</v>
       </c>
       <c r="F114" s="1" t="s">
         <v>198</v>
@@ -5773,19 +5776,19 @@
     </row>
     <row r="115">
       <c r="A115" s="1" t="s">
-        <v>230</v>
+        <v>78</v>
       </c>
       <c r="B115" s="1" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="C115" s="1" t="s">
         <v>63</v>
       </c>
       <c r="D115" s="5">
-        <v>0.6666666666666666</v>
+        <v>0.5</v>
       </c>
       <c r="E115" s="5">
-        <v>0.7916666666666666</v>
+        <v>0.5833333333333334</v>
       </c>
       <c r="F115" s="1" t="s">
         <v>198</v>
@@ -5793,82 +5796,122 @@
     </row>
     <row r="116">
       <c r="A116" s="1" t="s">
-        <v>231</v>
+        <v>82</v>
       </c>
       <c r="B116" s="1" t="s">
-        <v>232</v>
+        <v>228</v>
       </c>
       <c r="C116" s="1" t="s">
         <v>63</v>
       </c>
       <c r="D116" s="5">
-        <v>0.4166666666666667</v>
+        <v>0.5833333333333334</v>
       </c>
       <c r="E116" s="5">
-        <v>0.4548611111111111</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="F116" s="1" t="s">
-        <v>233</v>
+        <v>198</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="1" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="B117" s="1" t="s">
-        <v>232</v>
+        <v>228</v>
       </c>
       <c r="C117" s="1" t="s">
         <v>63</v>
       </c>
       <c r="D117" s="5">
-        <v>0.4583333333333333</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="E117" s="5">
-        <v>0.4791666666666667</v>
+        <v>0.7916666666666666</v>
       </c>
       <c r="F117" s="1" t="s">
-        <v>233</v>
+        <v>198</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="1" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="B118" s="1" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="C118" s="1" t="s">
         <v>63</v>
       </c>
       <c r="D118" s="5">
-        <v>0.4791666666666667</v>
+        <v>0.4166666666666667</v>
       </c>
       <c r="E118" s="5">
-        <v>0.5</v>
+        <v>0.4548611111111111</v>
       </c>
       <c r="F118" s="1" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="1" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="B119" s="1" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="C119" s="1" t="s">
         <v>63</v>
       </c>
       <c r="D119" s="5">
+        <v>0.4583333333333333</v>
+      </c>
+      <c r="E119" s="5">
+        <v>0.4791666666666667</v>
+      </c>
+      <c r="F119" s="1" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="1" t="s">
+        <v>236</v>
+      </c>
+      <c r="B120" s="1" t="s">
+        <v>233</v>
+      </c>
+      <c r="C120" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="D120" s="5">
+        <v>0.4791666666666667</v>
+      </c>
+      <c r="E120" s="5">
         <v>0.5</v>
       </c>
-      <c r="E119" s="5">
+      <c r="F120" s="1" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="B121" s="1" t="s">
+        <v>233</v>
+      </c>
+      <c r="C121" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="D121" s="5">
+        <v>0.5</v>
+      </c>
+      <c r="E121" s="5">
         <v>0.5833333333333334</v>
       </c>
-      <c r="F119" s="1" t="s">
-        <v>233</v>
+      <c r="F121" s="1" t="s">
+        <v>234</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add Saturday Wellness Village acts to timetable
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/The FullMoon Festival Linup.xlsx
+++ b/The FullMoon Festival Linup.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1220" uniqueCount="238">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1236" uniqueCount="238">
   <si>
     <t>THE FULLMOON FESTIVAL</t>
   </si>
@@ -5842,7 +5842,7 @@
         <v>233</v>
       </c>
       <c r="C118" s="1" t="s">
-        <v>63</v>
+        <v>48</v>
       </c>
       <c r="D118" s="5">
         <v>0.4166666666666667</v>
@@ -5862,7 +5862,7 @@
         <v>233</v>
       </c>
       <c r="C119" s="1" t="s">
-        <v>63</v>
+        <v>48</v>
       </c>
       <c r="D119" s="5">
         <v>0.4583333333333333</v>
@@ -5882,7 +5882,7 @@
         <v>233</v>
       </c>
       <c r="C120" s="1" t="s">
-        <v>63</v>
+        <v>48</v>
       </c>
       <c r="D120" s="5">
         <v>0.4791666666666667</v>
@@ -5902,7 +5902,7 @@
         <v>233</v>
       </c>
       <c r="C121" s="1" t="s">
-        <v>63</v>
+        <v>48</v>
       </c>
       <c r="D121" s="5">
         <v>0.5</v>
@@ -5911,6 +5911,86 @@
         <v>0.5833333333333334</v>
       </c>
       <c r="F121" s="1" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="B122" s="1" t="s">
+        <v>233</v>
+      </c>
+      <c r="C122" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="D122" s="5">
+        <v>0.4166666666666667</v>
+      </c>
+      <c r="E122" s="5">
+        <v>0.4548611111111111</v>
+      </c>
+      <c r="F122" s="1" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="1" t="s">
+        <v>235</v>
+      </c>
+      <c r="B123" s="1" t="s">
+        <v>233</v>
+      </c>
+      <c r="C123" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="D123" s="5">
+        <v>0.4583333333333333</v>
+      </c>
+      <c r="E123" s="5">
+        <v>0.4791666666666667</v>
+      </c>
+      <c r="F123" s="1" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="1" t="s">
+        <v>236</v>
+      </c>
+      <c r="B124" s="1" t="s">
+        <v>233</v>
+      </c>
+      <c r="C124" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="D124" s="5">
+        <v>0.4791666666666667</v>
+      </c>
+      <c r="E124" s="5">
+        <v>0.5</v>
+      </c>
+      <c r="F124" s="1" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="B125" s="1" t="s">
+        <v>233</v>
+      </c>
+      <c r="C125" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="D125" s="5">
+        <v>0.5</v>
+      </c>
+      <c r="E125" s="5">
+        <v>0.5833333333333334</v>
+      </c>
+      <c r="F125" s="1" t="s">
         <v>234</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update The Pub Friday acts and times
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/The FullMoon Festival Linup.xlsx
+++ b/The FullMoon Festival Linup.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1236" uniqueCount="238">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1236" uniqueCount="239">
   <si>
     <t>THE FULLMOON FESTIVAL</t>
   </si>
@@ -687,6 +687,9 @@
   </si>
   <si>
     <t>Band</t>
+  </si>
+  <si>
+    <t>Under The Bed</t>
   </si>
   <si>
     <t>The Pub</t>
@@ -5216,10 +5219,10 @@
     </row>
     <row r="87">
       <c r="A87" s="1" t="s">
-        <v>214</v>
+        <v>225</v>
       </c>
       <c r="B87" s="1" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C87" s="1" t="s">
         <v>29</v>
@@ -5228,7 +5231,7 @@
         <v>0.6354166666666666</v>
       </c>
       <c r="E87" s="5">
-        <v>0.65625</v>
+        <v>0.6875</v>
       </c>
       <c r="F87" s="1" t="s">
         <v>224</v>
@@ -5239,16 +5242,16 @@
         <v>146</v>
       </c>
       <c r="B88" s="1" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C88" s="1" t="s">
         <v>29</v>
       </c>
       <c r="D88" s="5">
-        <v>0.6770833333333334</v>
+        <v>0.7083333333333334</v>
       </c>
       <c r="E88" s="5">
-        <v>0.7395833333333334</v>
+        <v>0.7604166666666666</v>
       </c>
       <c r="F88" s="1" t="s">
         <v>224</v>
@@ -5259,16 +5262,16 @@
         <v>174</v>
       </c>
       <c r="B89" s="1" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C89" s="1" t="s">
         <v>29</v>
       </c>
       <c r="D89" s="5">
-        <v>0.7604166666666666</v>
+        <v>0.78125</v>
       </c>
       <c r="E89" s="5">
-        <v>0.8229166666666666</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="F89" s="1" t="s">
         <v>224</v>
@@ -5279,13 +5282,13 @@
         <v>176</v>
       </c>
       <c r="B90" s="1" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C90" s="1" t="s">
         <v>29</v>
       </c>
       <c r="D90" s="5">
-        <v>0.84375</v>
+        <v>0.8541666666666666</v>
       </c>
       <c r="E90" s="5">
         <v>0.90625</v>
@@ -5299,7 +5302,7 @@
         <v>177</v>
       </c>
       <c r="B91" s="1" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C91" s="1" t="s">
         <v>29</v>
@@ -5319,7 +5322,7 @@
         <v>169</v>
       </c>
       <c r="B92" s="1" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C92" s="1" t="s">
         <v>48</v>
@@ -5339,7 +5342,7 @@
         <v>149</v>
       </c>
       <c r="B93" s="1" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C93" s="1" t="s">
         <v>48</v>
@@ -5359,7 +5362,7 @@
         <v>182</v>
       </c>
       <c r="B94" s="1" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C94" s="1" t="s">
         <v>48</v>
@@ -5379,7 +5382,7 @@
         <v>184</v>
       </c>
       <c r="B95" s="1" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C95" s="1" t="s">
         <v>48</v>
@@ -5399,7 +5402,7 @@
         <v>186</v>
       </c>
       <c r="B96" s="1" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C96" s="1" t="s">
         <v>48</v>
@@ -5419,7 +5422,7 @@
         <v>187</v>
       </c>
       <c r="B97" s="1" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C97" s="1" t="s">
         <v>48</v>
@@ -5439,7 +5442,7 @@
         <v>188</v>
       </c>
       <c r="B98" s="1" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C98" s="1" t="s">
         <v>63</v>
@@ -5459,7 +5462,7 @@
         <v>153</v>
       </c>
       <c r="B99" s="1" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C99" s="1" t="s">
         <v>63</v>
@@ -5479,7 +5482,7 @@
         <v>148</v>
       </c>
       <c r="B100" s="1" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C100" s="1" t="s">
         <v>63</v>
@@ -5499,7 +5502,7 @@
         <v>160</v>
       </c>
       <c r="B101" s="1" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C101" s="1" t="s">
         <v>63</v>
@@ -5516,10 +5519,10 @@
     </row>
     <row r="102">
       <c r="A102" s="1" t="s">
+        <v>227</v>
+      </c>
+      <c r="B102" s="1" t="s">
         <v>226</v>
-      </c>
-      <c r="B102" s="1" t="s">
-        <v>225</v>
       </c>
       <c r="C102" s="1" t="s">
         <v>63</v>
@@ -5536,10 +5539,10 @@
     </row>
     <row r="103">
       <c r="A103" s="1" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B103" s="1" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C103" s="1" t="s">
         <v>29</v>
@@ -5559,7 +5562,7 @@
         <v>80</v>
       </c>
       <c r="B104" s="1" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C104" s="1" t="s">
         <v>29</v>
@@ -5576,10 +5579,10 @@
     </row>
     <row r="105">
       <c r="A105" s="1" t="s">
+        <v>230</v>
+      </c>
+      <c r="B105" s="1" t="s">
         <v>229</v>
-      </c>
-      <c r="B105" s="1" t="s">
-        <v>228</v>
       </c>
       <c r="C105" s="1" t="s">
         <v>29</v>
@@ -5599,7 +5602,7 @@
         <v>81</v>
       </c>
       <c r="B106" s="1" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C106" s="1" t="s">
         <v>29</v>
@@ -5619,7 +5622,7 @@
         <v>76</v>
       </c>
       <c r="B107" s="1" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C107" s="1" t="s">
         <v>29</v>
@@ -5639,7 +5642,7 @@
         <v>73</v>
       </c>
       <c r="B108" s="1" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C108" s="1" t="s">
         <v>29</v>
@@ -5659,7 +5662,7 @@
         <v>77</v>
       </c>
       <c r="B109" s="1" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C109" s="1" t="s">
         <v>29</v>
@@ -5679,7 +5682,7 @@
         <v>73</v>
       </c>
       <c r="B110" s="1" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C110" s="1" t="s">
         <v>48</v>
@@ -5699,7 +5702,7 @@
         <v>82</v>
       </c>
       <c r="B111" s="1" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C111" s="1" t="s">
         <v>48</v>
@@ -5719,7 +5722,7 @@
         <v>81</v>
       </c>
       <c r="B112" s="1" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C112" s="1" t="s">
         <v>48</v>
@@ -5739,7 +5742,7 @@
         <v>78</v>
       </c>
       <c r="B113" s="1" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C113" s="1" t="s">
         <v>48</v>
@@ -5756,10 +5759,10 @@
     </row>
     <row r="114">
       <c r="A114" s="1" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="B114" s="1" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C114" s="1" t="s">
         <v>48</v>
@@ -5779,7 +5782,7 @@
         <v>78</v>
       </c>
       <c r="B115" s="1" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C115" s="1" t="s">
         <v>63</v>
@@ -5799,7 +5802,7 @@
         <v>82</v>
       </c>
       <c r="B116" s="1" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C116" s="1" t="s">
         <v>63</v>
@@ -5816,10 +5819,10 @@
     </row>
     <row r="117">
       <c r="A117" s="1" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="B117" s="1" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C117" s="1" t="s">
         <v>63</v>
@@ -5836,10 +5839,10 @@
     </row>
     <row r="118">
       <c r="A118" s="1" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="B118" s="1" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="C118" s="1" t="s">
         <v>48</v>
@@ -5851,15 +5854,15 @@
         <v>0.4548611111111111</v>
       </c>
       <c r="F118" s="1" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="1" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="B119" s="1" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="C119" s="1" t="s">
         <v>48</v>
@@ -5871,15 +5874,15 @@
         <v>0.4791666666666667</v>
       </c>
       <c r="F119" s="1" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="1" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="B120" s="1" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="C120" s="1" t="s">
         <v>48</v>
@@ -5891,15 +5894,15 @@
         <v>0.5</v>
       </c>
       <c r="F120" s="1" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="1" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="B121" s="1" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="C121" s="1" t="s">
         <v>48</v>
@@ -5911,15 +5914,15 @@
         <v>0.5833333333333334</v>
       </c>
       <c r="F121" s="1" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="1" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="B122" s="1" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="C122" s="1" t="s">
         <v>63</v>
@@ -5931,15 +5934,15 @@
         <v>0.4548611111111111</v>
       </c>
       <c r="F122" s="1" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="1" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="B123" s="1" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="C123" s="1" t="s">
         <v>63</v>
@@ -5951,15 +5954,15 @@
         <v>0.4791666666666667</v>
       </c>
       <c r="F123" s="1" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="1" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="B124" s="1" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="C124" s="1" t="s">
         <v>63</v>
@@ -5971,15 +5974,15 @@
         <v>0.5</v>
       </c>
       <c r="F124" s="1" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="1" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="B125" s="1" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="C125" s="1" t="s">
         <v>63</v>
@@ -5991,7 +5994,7 @@
         <v>0.5833333333333334</v>
       </c>
       <c r="F125" s="1" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
     </row>
   </sheetData>

</xml_diff>